<commit_message>
Registration card on the event Overview
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-64_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-64_Test_Cases.xlsx
@@ -2547,7 +2547,7 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Event: SPM64 Closed Registration Seminar (Confirmed, starts 10 Mar 2027, 09:00) | Closes: 30 Sep 2026, 17:00 (already past) -&gt; 28 Feb 2027, 17:00</t>
+          <t>Event: SPM64 Closed Registration Seminar (Confirmed, starts 10 Mar 2027, 09:00) | Closes: 30 Sept 2026, 17:00 (already past) -&gt; 28 Feb 2027, 17:00</t>
         </is>
       </c>
     </row>
@@ -2559,7 +2559,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 1: The card shows 'Closes: 30 Sep 2026, 17:00', a date that has already passed.
+          <t>Step 1: The card shows 'Closes: 30 Sept 2026, 17:00', a date that has already passed.
 Step 4: 'Registration settings saved.' appears. The card shows 'Opens: 1 Aug 2026, 09:00' and 'Closes: 28 Feb 2027, 17:00'. The status badge still reads 'Confirmed'.</t>
         </is>
       </c>
@@ -4202,7 +4202,7 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Events: SPM64 Twin Room Workshop (registration off), SPM64 Closed Registration Seminar (on, capacity 50, 1 Aug 2026 09:00 – 30 Sep 2026 17:00) | Organiser: Evelyn Chen | Colleague: Raj Kumar (Straits Medical Institute)</t>
+          <t>Events: SPM64 Twin Room Workshop (registration off), SPM64 Closed Registration Seminar (on, capacity 50, 1 Aug 2026 09:00 – 30 Sept 2026 17:00) | Organiser: Evelyn Chen | Colleague: Raj Kumar (Straits Medical Institute)</t>
         </is>
       </c>
     </row>
@@ -4215,7 +4215,7 @@
       <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Step 1: The Registration card shows 'Registration: Not enabled for this event' and no 'Change registration settings' button.
-Step 2: The card shows 'Registration: Enabled', 'Capacity: 50', 'Measured against: Orchard Seminar Room (ORC-SEM), Classroom layout – up to 70', 'Opens: 1 Aug 2026, 09:00' and 'Closes: 30 Sep 2026, 17:00', with no 'Change registration settings' button.
+Step 2: The card shows 'Registration: Enabled', 'Capacity: 50', 'Measured against: Orchard Seminar Room (ORC-SEM), Classroom layout – up to 70', 'Opens: 1 Aug 2026, 09:00' and 'Closes: 30 Sept 2026, 17:00', with no 'Change registration settings' button.
 Step 4: The same values as in step 2, with no 'Change registration settings' button.</t>
         </is>
       </c>
@@ -4702,7 +4702,7 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Event: SPM64 Closed Registration Seminar (Confirmed, no registrations) | Capacity 50 | Opens 1 Aug 2026, 09:00 | Closes 30 Sep 2026, 17:00</t>
+          <t>Event: SPM64 Closed Registration Seminar (Confirmed, no registrations) | Capacity 50 | Opens 1 Aug 2026, 09:00 | Closes 30 Sept 2026, 17:00</t>
         </is>
       </c>
     </row>
@@ -4714,9 +4714,9 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 1: The card shows 'Registration: Enabled', 'Capacity: 50', 'Opens: 1 Aug 2026, 09:00' and 'Closes: 30 Sep 2026, 17:00'.
+          <t>Step 1: The card shows 'Registration: Enabled', 'Capacity: 50', 'Opens: 1 Aug 2026, 09:00' and 'Closes: 30 Sept 2026, 17:00'.
 Step 4: 'Registration settings saved.' appears, the card shows 'Registration: Not enabled for this event', and no 'Flagged for review' list is shown (nobody holds a place). The status badge still reads 'Confirmed'.
-Step 6: 'Registration capacity' shows 50, 'Registration opens' 1 Aug 2026 09:00 and 'Registration closes' 30 Sep 2026 17:00.
+Step 6: 'Registration capacity' shows 50, 'Registration opens' 1 Aug 2026 09:00 and 'Registration closes' 30 Sept 2026 17:00.
 Step 7: The card shows 'Registration: Enabled', 'Capacity: 50' and the same opening and closing times as in step 1.</t>
         </is>
       </c>

</xml_diff>